<commit_message>
modif tableau de synthese
</commit_message>
<xml_diff>
--- a/tableau_synthese1_2025.xlsx
+++ b/tableau_synthese1_2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\Portfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6AB96AD7-13BB-4F06-A8C1-F65741A50706}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F5384881-C3CE-495E-BB4E-FDB3577AA4FF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="820" yWindow="500" windowWidth="19740" windowHeight="12460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -122,9 +122,6 @@
     <t>Installation et configuration d'un serveur Linux virtualisé avec la gestion des incidents GLPI</t>
   </si>
   <si>
-    <t>Conception et développement du site internet E-Ensiegnement avec le CMS WordPresse</t>
-  </si>
-  <si>
     <t>Réalisations en milieu professionnel en cours de première année</t>
   </si>
   <si>
@@ -134,15 +131,9 @@
     <t>NOM et prénom :BOURAIMA IMDAD SAMORY AKANNI</t>
   </si>
   <si>
-    <t>Développement du jeu Snake en Langage C avec Git_GitHub en mode projet</t>
-  </si>
-  <si>
     <t xml:space="preserve">Centre de formation : IRIS </t>
   </si>
   <si>
-    <t>Formation Certification en:Node.js,SQL,ANSSI</t>
-  </si>
-  <si>
     <t>Nov 2025 a Fév 2026</t>
   </si>
   <si>
@@ -165,6 +156,15 @@
   </si>
   <si>
     <t>Adresse URL Portfolio : https://sp-bts-2026.github.io/portfolio_Bouraima/</t>
+  </si>
+  <si>
+    <t>Formation Certification en:Node.js,,ANSSI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conception et développement du site internet Legal help </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Développement d'un site ASIH de covoiturage et de taxi </t>
   </si>
 </sst>
 </file>
@@ -275,7 +275,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="27">
+  <borders count="32">
     <border>
       <left/>
       <right/>
@@ -613,6 +613,63 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color theme="2" tint="-0.749992370372631"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color theme="2" tint="-0.749992370372631"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="2" tint="-0.749992370372631"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </top>
+      <bottom style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color theme="2" tint="-0.749992370372631"/>
+      </right>
+      <top style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </top>
+      <bottom style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -620,7 +677,7 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -691,9 +748,36 @@
     <xf numFmtId="17" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -721,41 +805,23 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1078,56 +1144,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24" t="s">
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="24"/>
+      <c r="H1" s="25"/>
     </row>
     <row r="2" spans="1:43" ht="41.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
     </row>
     <row r="3" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="25" t="s">
-        <v>25</v>
-      </c>
-      <c r="B3" s="26"/>
-      <c r="C3" s="26"/>
-      <c r="D3" s="26"/>
-      <c r="E3" s="27"/>
-      <c r="F3" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="G3" s="32"/>
-      <c r="H3" s="33"/>
+      <c r="A3" s="34" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="35"/>
+      <c r="C3" s="35"/>
+      <c r="D3" s="35"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="40" t="s">
+        <v>32</v>
+      </c>
+      <c r="G3" s="41"/>
+      <c r="H3" s="42"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="B4" s="29"/>
-      <c r="C4" s="29"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="30"/>
+      <c r="A4" s="37" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="38"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="39"/>
       <c r="F4" s="7" t="s">
         <v>3</v>
       </c>
@@ -1139,22 +1205,22 @@
       </c>
     </row>
     <row r="5" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="B5" s="44"/>
-      <c r="C5" s="44"/>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="44"/>
-      <c r="G5" s="44"/>
-      <c r="H5" s="45"/>
+      <c r="A5" s="31" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="32"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="32"/>
+      <c r="H5" s="33"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="34" t="s">
+      <c r="A6" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="41" t="s">
+      <c r="B6" s="29" t="s">
         <v>7</v>
       </c>
       <c r="C6" s="10" t="s">
@@ -1177,8 +1243,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="325" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="34"/>
-      <c r="B7" s="42"/>
+      <c r="A7" s="24"/>
+      <c r="B7" s="30"/>
       <c r="C7" s="19" t="s">
         <v>14</v>
       </c>
@@ -1234,16 +1300,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A8" s="35" t="s">
+      <c r="A8" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="36"/>
-      <c r="C8" s="36"/>
-      <c r="D8" s="36"/>
-      <c r="E8" s="36"/>
-      <c r="F8" s="36"/>
-      <c r="G8" s="36"/>
-      <c r="H8" s="37"/>
+      <c r="B8" s="27"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="28"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1331,12 +1397,11 @@
     </row>
     <row r="10" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="B10" s="15">
         <v>45901</v>
       </c>
-      <c r="C10" s="12"/>
       <c r="D10" s="5"/>
       <c r="E10" s="13"/>
       <c r="F10" s="13"/>
@@ -1380,14 +1445,14 @@
     </row>
     <row r="11" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="B11" s="15">
         <v>45931</v>
       </c>
       <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="13"/>
       <c r="F11" s="13"/>
       <c r="G11" s="13"/>
       <c r="H11" s="6"/>
@@ -1425,14 +1490,13 @@
       <c r="AN11"/>
       <c r="AO11"/>
       <c r="AP11"/>
-      <c r="AQ11"/>
     </row>
     <row r="12" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
@@ -1478,7 +1542,7 @@
     </row>
     <row r="13" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B13" s="15">
         <v>45689</v>
@@ -1527,7 +1591,7 @@
     </row>
     <row r="14" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B14" s="18">
         <v>45597</v>
@@ -1576,14 +1640,14 @@
     </row>
     <row r="15" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B15" s="18">
         <v>45992</v>
       </c>
       <c r="C15" s="5"/>
       <c r="D15" s="13"/>
-      <c r="E15" s="5"/>
+      <c r="E15" s="13"/>
       <c r="F15" s="13"/>
       <c r="G15" s="13"/>
       <c r="H15" s="6"/>
@@ -1624,16 +1688,16 @@
       <c r="AQ15"/>
     </row>
     <row r="16" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A16" s="38" t="s">
-        <v>23</v>
-      </c>
-      <c r="B16" s="39"/>
-      <c r="C16" s="39"/>
-      <c r="D16" s="39"/>
-      <c r="E16" s="39"/>
-      <c r="F16" s="39"/>
-      <c r="G16" s="39"/>
-      <c r="H16" s="40"/>
+      <c r="A16" s="46" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" s="47"/>
+      <c r="C16" s="47"/>
+      <c r="D16" s="47"/>
+      <c r="E16" s="47"/>
+      <c r="F16" s="47"/>
+      <c r="G16" s="47"/>
+      <c r="H16" s="48"/>
       <c r="I16"/>
       <c r="J16"/>
       <c r="K16"/>
@@ -1672,10 +1736,10 @@
     </row>
     <row r="17" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B17" s="17"/>
-      <c r="C17" s="17"/>
+      <c r="C17" s="12"/>
       <c r="D17" s="5"/>
       <c r="E17" s="13"/>
       <c r="F17" s="5"/>
@@ -1763,16 +1827,16 @@
       <c r="AQ18"/>
     </row>
     <row r="19" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A19" s="38" t="s">
-        <v>24</v>
-      </c>
-      <c r="B19" s="39"/>
-      <c r="C19" s="39"/>
-      <c r="D19" s="39"/>
-      <c r="E19" s="39"/>
-      <c r="F19" s="39"/>
-      <c r="G19" s="39"/>
-      <c r="H19" s="40"/>
+      <c r="A19" s="43" t="s">
+        <v>23</v>
+      </c>
+      <c r="B19" s="44"/>
+      <c r="C19" s="44"/>
+      <c r="D19" s="44"/>
+      <c r="E19" s="44"/>
+      <c r="F19" s="44"/>
+      <c r="G19" s="44"/>
+      <c r="H19" s="45"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1811,11 +1875,11 @@
     </row>
     <row r="20" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B20" s="3"/>
       <c r="C20" s="5"/>
-      <c r="D20" s="17"/>
+      <c r="D20" s="13"/>
       <c r="E20" s="13"/>
       <c r="F20" s="13"/>
       <c r="G20" s="5"/>
@@ -1904,18 +1968,18 @@
     <row r="66" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A19:H19"/>
     <mergeCell ref="A16:H16"/>
-    <mergeCell ref="A19:H19"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="A5:H5"/>
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="F3:H3"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="A5:H5"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -1944,6 +2008,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="191d0fcf-6d89-4c90-807a-10f37b8d7a4c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9a7dc87b-2be1-4fee-871a-355a79ca984c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F136CB4AE69C04489071CEF15422A7D7" ma:contentTypeVersion="10" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="886fd2e30fa2cc1fdb685626e6ee64a7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="191d0fcf-6d89-4c90-807a-10f37b8d7a4c" xmlns:ns3="9a7dc87b-2be1-4fee-871a-355a79ca984c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4d458b4e84b684dffe91b93afc291e76" ns2:_="" ns3:_="">
     <xsd:import namespace="191d0fcf-6d89-4c90-807a-10f37b8d7a4c"/>
@@ -2132,17 +2207,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="191d0fcf-6d89-4c90-807a-10f37b8d7a4c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9a7dc87b-2be1-4fee-871a-355a79ca984c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{12891FC5-B985-42D8-BB15-5428EFF482F5}">
   <ds:schemaRefs>
@@ -2152,6 +2216,23 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B4B2C3C2-98C5-40C9-936C-A0749252C73F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="191d0fcf-6d89-4c90-807a-10f37b8d7a4c"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="9a7dc87b-2be1-4fee-871a-355a79ca984c"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{115E9D4D-BBFA-4016-A3EB-D1328016C37C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2168,21 +2249,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B4B2C3C2-98C5-40C9-936C-A0749252C73F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="9a7dc87b-2be1-4fee-871a-355a79ca984c"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="191d0fcf-6d89-4c90-807a-10f37b8d7a4c"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>